<commit_message>
Expand Hamburg designer job-lead list from 12 to 19 companies
Add 7 further Hamburg employers currently advertising graphic/media
designer roles across new sectors (publishing, fashion/retail,
agencies, gastronomy outfitter): Carlsen Verlag, HINSCHE Gastrowelt,
Saint Elmo's, fischerAppelt, Mutabor, TOM TAILOR, UNGER Fashion.
Contact data sourced from company imprints / commercial register.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WaUcRs54TqxPzss59GmsGY
</commit_message>
<xml_diff>
--- a/Leads_Hamburg_Grafiker_Mediengestalter.xlsx
+++ b/Leads_Hamburg_Grafiker_Mediengestalter.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Hinweise &amp; Methodik" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads Hamburg'!$A$4:$N$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Leads Hamburg'!$A$4:$N$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1469,8 +1469,498 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="78" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Carlsen Verlag GmbH</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Mediengestalter:in / Mediendesign (Digital &amp; Print)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Gestaltung/Reinzeichnung von Buch-, Marketing- und Digitalmedien; teils Homeoffice moeglich.</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Ausbildung/Studium Mediengestaltung/Kommunikationsdesign; Adobe InDesign/Photoshop/Illustrator.</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Buchverlag (Kinder-/Jugendbuch, Comics/Manga; Bonnier-Gruppe). Sitz Ottensen.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Verlag stellt lfd. ein, teils befristet</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Bewerbung ueber Karriereportal</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>ueber carlsen.de/karriere</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>+49 40 39804-0</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Voelckersstr. 14-20, 22765 Hamburg-Ottensen</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>www.carlsen.de</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>StepStone / dasauge</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="78" customHeight="1">
+      <c r="A18" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>HINSCHE Gastrowelt GmbH</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Mediengestalter (m/w/d) Digital und Print</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Konzeption/Gestaltung von Print- &amp; Werbematerialien (Flyer, Kataloge, Anzeigen, Plakate, Geschaeftsausstattung); Support Digital &amp; Social Media.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Ausbildung Mediengestalter Digital und Print; Adobe Creative Suite.</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Gastro-Gesamtausstatter (Gastronomie/Hotellerie/Grosskueche, &gt;85 J.). Standort Hamburg; HR-Sitz Oldenburg.</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>Standort HH, Recruiting ueber Zentrale</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Sebastian Pozo (Personalabteilung)</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>bewerbung@hinsche-gastrowelt.de</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>+49 441 9355-234</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Standort Hamburg; HR: Wilhelmshavener Heerstr. 65, 26125 Oldenburg</t>
+        </is>
+      </c>
+      <c r="M18" s="10" t="inlineStr">
+        <is>
+          <t>www.hinsche-gastrowelt.de</t>
+        </is>
+      </c>
+      <c r="N18" s="9" t="inlineStr">
+        <is>
+          <t>hamburger.jobs / heyjobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="78" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Saint Elmo's Hamburg GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Mediengestalter / Reinzeichner (all genders)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Reinzeichnung/Gestaltung fuer Print &amp; Digital in einer Kreativ-/Werbeagentur.</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Ausbildung Mediengestalter/Reinzeichner; sicher in Adobe.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Kreativ-/Werbeagentur (Saint Elmo's Group). GF Peter Gocht (HRA 118172).</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Agentur, laufend im Recruiting</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Peter Gocht (Managing Director)</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>ueber saint-elmos.com (Impressum)</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>+49 40 2022888302</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Steinhoeft 9, 20459 Hamburg</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>www.saint-elmos.com</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>Indeed / trabajo.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="78" customHeight="1">
+      <c r="A20" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>fischerAppelt AG</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Mediengestalter:in / Grafiker:in (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Gestaltung/Reinzeichnung fuer Content-, PR- und Digitalprojekte.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Ausbildung/Studium Grafik/Mediengestaltung; Adobe; crossmediales Arbeiten.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Fuehrende Content-Marketing- &amp; PR-Agenturgruppe. Vorstand B. &amp; A. Fischer-Appelt (HRB 77749).</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>grosse Agentur, mehrere Kreativ-Rollen offen</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>kein Name genannt</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>info@fischerappelt.de</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>+49 40 899699-0</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Waterloohain 5, 22769 Hamburg-Eimsbuettel</t>
+        </is>
+      </c>
+      <c r="M20" s="10" t="inlineStr">
+        <is>
+          <t>www.fischerappelt.com</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>dasauge / trabajo.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Mutabor Design GmbH</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Mediengestalter:in / Grafiker:in (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Gestaltung/Umsetzung von Markenauftritten (Brand Design, Kampagnen, Retail/Environmental).</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Ausbildung/Studium Grafik-/Kommunikationsdesign; Adobe CC.</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Renommierte Markenagentur (Strategy, Design &amp; Technology). GF Paravicini, Plass, Breid (HRB 81512).</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>renommierte Agentur, lfd. Designbedarf</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>kein Name genannt</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>ueber mutabor.com/contact</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>040 39922410</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Grosse Elbstrasse 145b, 22767 Hamburg-Altona</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>www.mutabor.com</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>dasauge / designmadeingermany</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>TOM TAILOR GmbH</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>(Junior/Senior) Graphic Designer (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Erstellung CI-basierter Online- &amp; Print-Assets; Plakate, Inlays, Anzeigen; Praesentationen &amp; Guidelines. Hybrid.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Ausbildung/Studium Grafik/Mediengestaltung; Adobe; Fashion-/Brand-Affinitaet.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Casual-Fashion- &amp; Lifestyle-Marke. Sitz Hamburg (Norderstedt/Garstedter Weg).</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>Junior UND Senior parallel gesucht</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Bewerbung ueber Stellenmarkt (tom-tailor.de)</t>
+        </is>
+      </c>
+      <c r="J22" s="10" t="inlineStr">
+        <is>
+          <t>info@tom-tailor.com</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>+49 40 58956-0</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Garstedter Weg 14, 22453 Hamburg</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>company.tom-tailor.com</t>
+        </is>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>tom-tailor.de / trabajo.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="78" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>UNGER GmbH &amp; Co. KG (UNGER Fashion)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Kommunikationsdesigner (m/w/d), Voll-/Teilzeit</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Grafik, Reinzeichnung, Design fuer Store &amp; Onlineshop; Qualitaetskontrolle der Darstellung.</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Ausbildung/Studium Grafik/Kommunikationsdesign; Adobe; E-Commerce-Affinitaet.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Luxus-Mode: Store am Neuer Wall + internationaler Onlineshop (&gt;150 Marken, &gt;140 J.). GF Florian Braun.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>laufend 2026</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>breites Profil (Grafik + Reinzeichnung + QA)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>kein Name genannt</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>ueber unger-fashion.com/kontakt</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>s. Website</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Neuer Wall 35, 20354 Hamburg</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>www.unger-fashion.com</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>Indeed / dasauge</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:N16"/>
+  <autoFilter ref="A4:N23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId2"/>
@@ -1495,6 +1985,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M23" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>